<commit_message>
Card effect changes. Changed how skill card works. They now replace existing avatar cards. Avatar cards is  a token card which can be played at any time at the cost of MP.
</commit_message>
<xml_diff>
--- a/sheet/EventCardData.xlsx
+++ b/sheet/EventCardData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\nanDeck\DungeonCrawlDeckMaster\sheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEFD5B52-5C1A-4DB9-B317-F10A71526DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEF96F13-1EFC-40C3-BA01-293D74EFC77D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5595" yWindow="2910" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>cardName</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -225,6 +225,30 @@
   </si>
   <si>
     <t>多选：①可重复，支付3金币，从购买能力区选1张牌获得。②可重复至多3次，支付1金币，将购买能力区补满，然后重抽其中任意张牌。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>泉水</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回复一半MP（向下取整）。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>采石场</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>消耗1时间，从遭遇牌堆翻开前2张《水晶》或《金块》，加入背包区。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>废弃营地</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>消耗1时间，从遭遇牌堆翻开前2张《木柴捆》，加入背包区。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -574,7 +598,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="32.125" customWidth="1"/>
@@ -678,42 +702,86 @@
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
     </row>
-    <row r="7" spans="1:6" ht="57" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+    </row>
+    <row r="8" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+    </row>
+    <row r="9" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="C10" s="1"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+    </row>
+    <row r="11" spans="1:6" ht="57" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="71.25" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+    <row r="12" spans="1:6" ht="71.25" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>23</v>
       </c>
-      <c r="B8">
-        <v>2</v>
-      </c>
-      <c r="C8" s="1" t="s">
+      <c r="B12">
+        <v>2</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E12" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="57" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+    <row r="13" spans="1:6" ht="57" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>25</v>
       </c>
-      <c r="B9">
-        <v>2</v>
-      </c>
-      <c r="C9" s="1" t="s">
+      <c r="B13">
+        <v>2</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>29</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add time consuming related effects to some event cards. Add Ammo Pouch Item card which can put some Ammo cards in. Update rulebook adding minor change on positioning of room sides.
</commit_message>
<xml_diff>
--- a/sheet/EventCardData.xlsx
+++ b/sheet/EventCardData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\nanDeck\DungeonCrawlDeckMaster\sheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEF96F13-1EFC-40C3-BA01-293D74EFC77D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E1E0DF0-C66D-46A1-BA1F-D95B23633D9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5595" yWindow="2910" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>cardName</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -171,15 +171,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>地下城重整</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>重抽场上所有敌人侧的牌。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>翻开遭遇牌堆前3张牌，获得其中1张物品牌。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -224,31 +216,48 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>多选：①可重复，支付3金币，从购买能力区选1张牌获得。②可重复至多3次，支付1金币，将购买能力区补满，然后重抽其中任意张牌。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>泉水</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>回复一半MP（向下取整）。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>采石场</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>消耗1时间，从遭遇牌堆翻开前2张《水晶》或《金块》，加入背包区。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>废弃营地</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>消耗1时间，从遭遇牌堆翻开前2张《木柴捆》，加入背包区。</t>
+    <t>重组</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>从遭遇牌堆翻开第1张《金块》，加入背包区，再消耗1时间，可以重复1次该效果。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>从遭遇牌堆翻开第1张《木柴捆》，加入背包区，再消耗1时间，可以重复1次该效果。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回复一半MP（向下取整）。&lt;br&gt;
+消耗1时间，从遭遇牌堆翻开第1张《魔瓶》，加入背包区。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>弹药堆</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>从遭遇牌堆翻开前2张“弹药”牌，加入背包区，再消耗1时间，可以重复1次该效果。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>翻开遭遇牌堆前3张牌，获得其中1张物品牌，再消耗1时间，可以重复1次该效果。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>多选：①可重复，支付3金币，从购买能力区选1张牌获得。②可重复，支付1金币，将购买能力区补满，然后重抽其中任意张牌，每次重复该效果，需要支付的金币数量加1。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -627,13 +636,13 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="B2">
-        <v>2</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>2</v>
@@ -642,7 +651,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -650,20 +659,20 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:6" ht="92.25" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B4">
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>3</v>
@@ -674,13 +683,13 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B5">
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>4</v>
@@ -691,58 +700,66 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
     </row>
-    <row r="8" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B8">
         <v>2</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
     </row>
-    <row r="9" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B9">
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C10" s="1"/>
+    <row r="10" spans="1:6" ht="42.75" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>35</v>
+      </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
     </row>
@@ -754,18 +771,18 @@
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B12">
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>5</v>
@@ -774,15 +791,15 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="57" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B13">
         <v>2</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Card description change: Splash slime, Bless, Curse, Tome, Unknown scroll, Shop. Card effect change: Ammo stash -> now grant 1 ammo card instead of 2. Dream catcher -> Only redraw cards in the field. Add card: Fast deployment -> Passive. Allow player to play cards at the start of turn start. Liquidation -> Passive. Allow player to discard an item card at any time and get 1 gold for each card discarded this way. Recycle -> Passive. Each time an item card is discarded, get 1 gold. Bar -> Event. Pay 3 gold to draw 1 card. Update rulebook: Add rule description on ammo cards -> They are used by an avatar card in the field. Add rules on factions. Add keyword Sell.
</commit_message>
<xml_diff>
--- a/sheet/EventCardData.xlsx
+++ b/sheet/EventCardData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\nanDeck\DungeonCrawlDeckMaster\sheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E1E0DF0-C66D-46A1-BA1F-D95B23633D9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{441B6264-D8A8-41D3-BEE2-0B827E6C74BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5595" yWindow="2910" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3075" yWindow="3075" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t>cardName</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -171,10 +171,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>重抽场上所有敌人侧的牌。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>拉杆</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -195,11 +191,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>多选：①弃置1张物品牌。②将1张手牌送墓。③受到2伤害。&lt;br&gt;
-执行2项以上时：从购买能力区选1张牌获得。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>训练场</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -209,10 +200,6 @@
   </si>
   <si>
     <t>将弃牌堆顶的1张牌放回主牌堆。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>多选：①可重复至多3次，弃置1张物品牌，然后获得1金币。②取遭遇牌堆前3张物品牌，然后玩家每支付2金币，可以获得其中1张牌。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -249,15 +236,36 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>从遭遇牌堆翻开前2张“弹药”牌，加入背包区，再消耗1时间，可以重复1次该效果。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>翻开遭遇牌堆前3张牌，获得其中1张物品牌，再消耗1时间，可以重复1次该效果。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>多选：①可重复，支付3金币，从购买能力区选1张牌获得。②可重复，支付1金币，将购买能力区补满，然后重抽其中任意张牌，每次重复该效果，需要支付的金币数量加1。</t>
+    <t>重抽场上所有地城阵营的牌。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>从遭遇牌堆翻开第1张“弹药”牌，加入背包区，再消耗1时间，可以重复1次该效果。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>多选：①弃置1张物品牌。②将1张手牌送墓。③受到1伤害。&lt;br&gt;
+执行2项以上时：从购买能力区选1张牌获得。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>多选：①可重复，出售1张物品牌并获得1金币。②取遭遇牌堆前3张物品牌，然后玩家每支付2金币，可以获得其中1张牌。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>酒馆</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>多选：①支付8金币，从购买升级区选1张牌获得。②可重复，支付3金币，将购买能力区补满，然后重抽其中任意张牌，每次重复该效果，需要支付的金币数量加1。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>可重复，支付3金币，抽1张牌。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -607,7 +615,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="32.125" customWidth="1"/>
@@ -636,13 +644,13 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B2">
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>2</v>
@@ -659,20 +667,20 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:6" ht="92.25" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="B4">
-        <v>2</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>18</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>3</v>
@@ -683,13 +691,13 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B5">
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>4</v>
@@ -700,65 +708,65 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:6" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
     </row>
     <row r="8" spans="1:6" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="B8">
-        <v>2</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
     </row>
     <row r="9" spans="1:6" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="B9">
-        <v>2</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>32</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
     </row>
     <row r="10" spans="1:6" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="B10">
-        <v>2</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>35</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
@@ -771,18 +779,18 @@
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B12">
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>5</v>
@@ -793,13 +801,24 @@
     </row>
     <row r="13" spans="1:6" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B13">
         <v>2</v>
       </c>
       <c r="C13" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>37</v>
+      </c>
+      <c r="B14">
+        <v>2</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Card effect change: Genocide -> pick a card at hand instead of claiming a race. Bar -> cost 5 gold per usage. Shop -> sell 1 item card for 2 gold (instead of 1) and buy 1 item card for 4 gold (instead of 3). Ammo box -> stack cards only when not tapped. take out cards only when tapped. can tap at any time. Card description change: Boulder -> use Survive keyword. Deck change: Reduce the cost of most spell cards. Add Shop cards from 2 copies to 3. Add Mule cards -> Passive. Add 1 capacity to backpack zone. Rule change: Half is always rounded up now. Player initially has 4 hp and 4 mp now. The player can only use bonus cards when there is no enemy cards( instead of no cards) in the corresponding row/column. Clarified "Move in/out". Clarified "Effect queue". Queued effects are invalidated if the card is not in the field when resolved.
</commit_message>
<xml_diff>
--- a/sheet/EventCardData.xlsx
+++ b/sheet/EventCardData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\nanDeck\DungeonCrawlDeckMaster\sheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{441B6264-D8A8-41D3-BEE2-0B827E6C74BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{436124DE-1835-4239-AEEA-0BCA9421FFD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3075" yWindow="3075" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -179,10 +179,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>获得遭遇牌堆第1张物品牌。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>宝箱</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -199,10 +195,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>将弃牌堆顶的1张牌放回主牌堆。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>泉水</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -227,45 +219,53 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>回复一半MP（向下取整）。&lt;br&gt;
+    <t>弹药堆</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>重抽场上所有地城阵营的牌。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>从遭遇牌堆翻开第1张“弹药”牌，加入背包区，再消耗1时间，可以重复1次该效果。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>酒馆</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>多选：①支付8金币，从购买升级区选1张牌获得。②可重复，支付3金币，将购买能力区补满，然后重抽其中任意张牌，每次重复该效果，需要支付的金币数量加1。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>可重复，支付5金币，抽1张牌。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回复一半MP。&lt;br&gt;
 消耗1时间，从遭遇牌堆翻开第1张《魔瓶》，加入背包区。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>弹药堆</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>翻开遭遇牌堆前3张牌，获得其中1张物品牌，再消耗1时间，可以重复1次该效果。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>重抽场上所有地城阵营的牌。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>从遭遇牌堆翻开第1张“弹药”牌，加入背包区，再消耗1时间，可以重复1次该效果。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>多选：①弃置1张物品牌。②将1张手牌送墓。③受到1伤害。&lt;br&gt;
+    <t>将弃牌堆顶的1张牌放在任意房间的地城侧。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>多选：①弃置1张道具牌。②将1张手牌送墓。③受到1伤害。&lt;br&gt;
 执行2项以上时：从购买能力区选1张牌获得。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>多选：①可重复，出售1张物品牌并获得1金币。②取遭遇牌堆前3张物品牌，然后玩家每支付2金币，可以获得其中1张牌。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>酒馆</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>多选：①支付8金币，从购买升级区选1张牌获得。②可重复，支付3金币，将购买能力区补满，然后重抽其中任意张牌，每次重复该效果，需要支付的金币数量加1。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>可重复，支付3金币，抽1张牌。</t>
+    <t>翻开遭遇牌堆前3张牌，获得其中1张道具牌，再消耗1时间，可以重复1次该效果。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>获得遭遇牌堆第1张道具牌。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>多选：①可重复，出售1张道具牌并获得1金币。②取遭遇牌堆前3张道具牌，然后玩家每支付3金币，可以获得其中1张牌。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -644,13 +644,13 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B2">
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>2</v>
@@ -667,7 +667,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
@@ -691,13 +691,13 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B5">
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>4</v>
@@ -706,67 +706,67 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:6" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
     </row>
     <row r="8" spans="1:6" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B8">
         <v>2</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
     </row>
     <row r="9" spans="1:6" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B9">
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
     </row>
     <row r="10" spans="1:6" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B10">
         <v>2</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
@@ -779,18 +779,18 @@
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>5</v>
@@ -801,24 +801,24 @@
     </row>
     <row r="13" spans="1:6" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B13">
         <v>2</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B14">
         <v>2</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Last commit has some changes unapplied. Fix that.
</commit_message>
<xml_diff>
--- a/sheet/EventCardData.xlsx
+++ b/sheet/EventCardData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\nanDeck\DungeonCrawlDeckMaster\sheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{436124DE-1835-4239-AEEA-0BCA9421FFD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A26AF7F-74F2-4932-B529-CD3E33167DCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2640" yWindow="2640" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -265,7 +265,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>多选：①可重复，出售1张道具牌并获得1金币。②取遭遇牌堆前3张道具牌，然后玩家每支付3金币，可以获得其中1张牌。</t>
+    <t>多选：①可重复，出售1张道具牌并获得2金币。②取遭遇牌堆前3张道具牌，然后玩家每支付4金币，可以获得其中1张牌。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>

</xml_diff>

<commit_message>
Removed card: Camp tools. Card effect change: Sentinel bot -> now rally a friendly monster from an adjacent room. Fuse slime -> now rally a slime monster from an adjacent rooms at turn end. Rally all slime monsters from all adjacent  rooms on battle start. Tomb -> now rally a monster from the top of the graveyard if there is a hostile card in its room on turn end. Rule change: Ammo cards  is now a standalone type. Ammo cards can also be used by any player-controlled monster cards with enough rank. All item cards and ammo cards can stack in player's inventory zone now. Add card type: Field card. They are cards with continuous effect and stays in bonus zone. They affect their territories, which is the corresponding row/column of their bonus zone. Changed the following former trap cards to field cards: Quicksand. Swamp. Cryo-gas vent. Add card: Ammo -> Confuse dart. Ammo -> Sleep dart. Ammo -> Canon ball. Field -> Altar. Card change: lowered the rank of some trap cards.
</commit_message>
<xml_diff>
--- a/sheet/EventCardData.xlsx
+++ b/sheet/EventCardData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\nanDeck\DungeonCrawlDeckMaster\sheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A26AF7F-74F2-4932-B529-CD3E33167DCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3306E39E-6F2E-40FE-BEB7-A87A6ADA6B9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2640" yWindow="2640" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>cardName</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -51,10 +51,6 @@
   </si>
   <si>
     <t>Lever</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Chest</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -138,19 +134,11 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>① Activate: Add the first two { Loot } cards from the Event Deck to your Loot Zone.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>① Activate, repeatable: Trade 2 non-gold resource for 1 gold or trade 1 gold for 1 non-gold resource. &lt;br&gt;
 ② Activate only when the Player does not have [Wanted] artifact card: Get 1 resource of each type. Then add a [Wanted] card from the Artifact Deck to your Equipment Zone.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>杂物堆</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>maxCount</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -167,18 +155,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>祭坛</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>拉杆</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>选场上1张陷阱牌，触发它或将其移动到场上任意位置。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>宝箱</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -191,81 +171,83 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>足迹</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>泉水</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>采石场</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>废弃营地</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>重组</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>从遭遇牌堆翻开第1张《金块》，加入背包区，再消耗1时间，可以重复1次该效果。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>从遭遇牌堆翻开第1张《木柴捆》，加入背包区，再消耗1时间，可以重复1次该效果。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>弹药堆</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>重抽场上所有地城阵营的牌。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>从遭遇牌堆翻开第1张“弹药”牌，加入背包区，再消耗1时间，可以重复1次该效果。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>酒馆</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>多选：①支付8金币，从购买升级区选1张牌获得。②可重复，支付3金币，将购买能力区补满，然后重抽其中任意张牌，每次重复该效果，需要支付的金币数量加1。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>可重复，支付5金币，抽1张牌。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>回复一半MP。&lt;br&gt;
-消耗1时间，从遭遇牌堆翻开第1张《魔瓶》，加入背包区。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>将弃牌堆顶的1张牌放在任意房间的地城侧。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>多选：①弃置1张道具牌。②将1张手牌送墓。③受到1伤害。&lt;br&gt;
-执行2项以上时：从购买能力区选1张牌获得。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>翻开遭遇牌堆前3张牌，获得其中1张道具牌，再消耗1时间，可以重复1次该效果。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>获得遭遇牌堆第1张道具牌。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>多选：①可重复，出售1张道具牌并获得2金币。②取遭遇牌堆前3张道具牌，然后玩家每支付4金币，可以获得其中1张牌。</t>
+    <t>图书馆</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回复一半MP。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>召唤石</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>将楼层区所有牌洗回对应牌堆，然后重置楼层区。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>选场上1张陷阱牌，将其移动到楼层区任意房间。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>地城重组</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>追踪足迹</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>金币堆</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>获得1金币。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>散落的金币</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>获得2金币。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>翻开升级牌堆前3张技能牌，获得其中1张。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>翻开升级牌堆前3张法术牌，获得其中1张。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>神龛</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>翻开升级牌堆前3张被动牌，获得其中1张。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>翻开主牌堆前3张怪物牌，选其中1张加入手牌。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>多选：①可重复，出售1张道具牌并获得1金币。②翻开遭遇牌堆前3张道具牌，然后玩家可以支付金币购买其中任意张道具牌，每支付2金币，获得其中1张道具牌。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>翻开遭遇牌堆前3张牌，获得其中所有道具牌和弹药牌。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -615,7 +597,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="32.125" customWidth="1"/>
@@ -627,179 +609,173 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
       </c>
       <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>13</v>
       </c>
-      <c r="F1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2">
-        <v>2</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="42.75" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
       <c r="B3">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:6" ht="92.25" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B4">
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B5">
         <v>2</v>
       </c>
-      <c r="C5" t="s">
-        <v>38</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="C5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
     </row>
-    <row r="7" spans="1:6" ht="42.75" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
     </row>
-    <row r="8" spans="1:6" ht="42.75" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="B8">
         <v>2</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
     </row>
-    <row r="9" spans="1:6" ht="42.75" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-    </row>
-    <row r="10" spans="1:6" ht="42.75" x14ac:dyDescent="0.2">
+        <v>34</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:6" ht="57" x14ac:dyDescent="0.2">
+      <c r="E10" s="3"/>
+    </row>
+    <row r="11" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>15</v>
       </c>
       <c r="B11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="71.25" x14ac:dyDescent="0.2">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="71.25" x14ac:dyDescent="0.2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -807,17 +783,6 @@
         <v>2</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>31</v>
-      </c>
-      <c r="B14">
-        <v>2</v>
-      </c>
-      <c r="C14" s="1" t="s">
         <v>33</v>
       </c>
     </row>

</xml_diff>